<commit_message>
Credited datasets and review sheet columns (phase 2, A3 and A4)
Adds data/credited/ with origins, videos, GI products, railway stations,
Wikidata IDs, and empty or one-row monuments, parishes and feasts files.
Village codes are matched by name and marked checked=no; ambiguous ones
are left blank. The review sheet gets gazetteer_devanagari,
advisory_body_form, gazetteer_page and luis_spelling. The build stops if
a credited village code is not an LGD code.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/village_names_review.xlsx
+++ b/data/village_names_review.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Review" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Review'!$A$1:$R$430</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Review'!$A$1:$V$430</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -536,7 +536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R430"/>
+  <dimension ref="A1:V430"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -557,6 +557,10 @@
     <col width="19" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
     <col width="15" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
+    <col width="22" customWidth="1" min="20" max="20"/>
+    <col width="22" customWidth="1" min="21" max="21"/>
+    <col width="22" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -650,6 +654,26 @@
           <t>Reviewer note</t>
         </is>
       </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>gazetteer_devanagari</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>advisory_body_form</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>gazetteer_page</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>luis_spelling</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -670,7 +694,6 @@
           <t>Agonda</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>DEVALKAJJAN</t>
@@ -726,7 +749,6 @@
           <t>Angediva</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>CHAURI</t>
@@ -772,7 +794,6 @@
           <t>Canacona</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -808,7 +829,6 @@
           <t>Chaudi</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -844,7 +864,6 @@
           <t>Cola</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>KOLA</t>
@@ -895,7 +914,6 @@
           <t>Cotigao</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>COTIGAO</t>
@@ -941,7 +959,6 @@
           <t>Gaodongrem</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>GAUNDONGREN</t>
@@ -987,7 +1004,6 @@
           <t>Loliem</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>LOLEN</t>
@@ -1038,7 +1054,6 @@
           <t>Nagorcem - Palolem</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -1074,7 +1089,6 @@
           <t>Poinguinim</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>POINGUNIN</t>
@@ -1120,7 +1134,6 @@
           <t>Aglote</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>AALOT</t>
@@ -1171,7 +1184,6 @@
           <t>Bandoli</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>BANDOLI</t>
@@ -1217,7 +1229,6 @@
           <t>Camarconda</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>KAMARKHAND</t>
@@ -1263,7 +1274,6 @@
           <t>Caranzol</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>KARANJHOL</t>
@@ -1309,7 +1319,6 @@
           <t>Codli</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>KODLI</t>
@@ -1355,7 +1364,6 @@
           <t>Colem</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>KOLEM</t>
@@ -1381,6 +1389,11 @@
       <c r="P17" s="2" t="n"/>
       <c r="Q17" s="2" t="n"/>
       <c r="R17" s="2" t="n"/>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>Kulem</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1401,7 +1414,6 @@
           <t>Cormonem</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -1437,7 +1449,6 @@
           <t>Darbandora</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>DARBANDORA</t>
@@ -1483,7 +1494,6 @@
           <t>Moissal</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>KAMARKHAND</t>
@@ -1529,7 +1539,6 @@
           <t>Molem</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>MOLEN</t>
@@ -1575,7 +1584,6 @@
           <t>Piliem</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
       <c r="L22" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -1611,7 +1619,6 @@
           <t>Sancordem</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>SAKVORDE</t>
@@ -1657,7 +1664,6 @@
           <t>Sangod</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>SANGOD</t>
@@ -1703,7 +1709,6 @@
           <t>Sigao</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>SHIGAON</t>
@@ -1749,7 +1754,6 @@
           <t>Sonauli</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>SONAULI</t>
@@ -1795,7 +1799,6 @@
           <t>Surla</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>SURLA</t>
@@ -1841,7 +1844,6 @@
           <t>Adnem</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>ADNE</t>
@@ -1892,7 +1894,6 @@
           <t>Ambaulim</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>AMBAVALI</t>
@@ -1943,7 +1944,6 @@
           <t>Amona</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
       <c r="L30" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -1979,7 +1979,6 @@
           <t>Assolda</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
           <t>ASOLDA</t>
@@ -2030,7 +2029,6 @@
           <t>Avedem</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
           <t>AVEDEN</t>
@@ -2081,7 +2079,6 @@
           <t>Bali</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
           <t>BALLY</t>
@@ -2132,7 +2129,6 @@
           <t>Barcem</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
           <t>BARSEN</t>
@@ -2183,7 +2179,6 @@
           <t>Bendordem</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
           <t>BENDODE</t>
@@ -2234,7 +2229,6 @@
           <t>Cacora</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -2270,7 +2264,6 @@
           <t>Cavorem</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -2306,7 +2299,6 @@
           <t>Cazur</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
           <t>BAMBUBOUTHAN</t>
@@ -2352,7 +2344,6 @@
           <t>Chaifi</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
           <t>CHAYAPHI</t>
@@ -2398,7 +2389,6 @@
           <t>Cordem</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
       <c r="L40" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -2434,7 +2424,6 @@
           <t>Corla</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
           <t>KARL  KAJUGATTO</t>
@@ -2480,7 +2469,6 @@
           <t>Cotombi</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
           <t>KAKODA</t>
@@ -2526,7 +2514,6 @@
           <t>Curchorem</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
       <c r="L43" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -2562,7 +2549,6 @@
           <t>Cusmane</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
       <c r="L44" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -2598,7 +2584,6 @@
           <t>Deao</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
       <c r="L45" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -2634,7 +2619,6 @@
           <t>Fatorpa</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
           <t>FATARPA</t>
@@ -2685,7 +2669,6 @@
           <t>Goculdem</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
           <t>GOKOLE</t>
@@ -2736,7 +2719,6 @@
           <t>Hodar</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
       <c r="L48" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -2772,7 +2754,6 @@
           <t>Maina</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
           <t>MAYNA</t>
@@ -2823,7 +2804,6 @@
           <t>Mangal</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
           <t>MANGAL</t>
@@ -2869,7 +2849,6 @@
           <t>Molcopona</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
         <is>
           <t>MALKAPOM</t>
@@ -2915,7 +2894,6 @@
           <t>Molcornem</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
           <t>MALKARNE</t>
@@ -2966,7 +2944,6 @@
           <t>Morpirla</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -3002,7 +2979,6 @@
           <t>Nagvem</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
         <is>
           <t>NAGVEM</t>
@@ -3048,7 +3024,6 @@
           <t>Naqueri</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
           <t>NAKERI</t>
@@ -3099,7 +3074,6 @@
           <t>Padi</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
           <t>PADI</t>
@@ -3150,7 +3124,6 @@
           <t>Pirla</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr">
         <is>
           <t>PIRL</t>
@@ -3201,7 +3174,6 @@
           <t>Quedem</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
         <is>
           <t>KHEDE</t>
@@ -3252,7 +3224,6 @@
           <t>Quepem</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
       <c r="L59" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -3288,7 +3259,6 @@
           <t>Quisconda</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
           <t>KISKON</t>
@@ -3334,7 +3304,6 @@
           <t>Quitol</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
           <t>KITAL</t>
@@ -3380,7 +3349,6 @@
           <t>Sirvoi</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
           <t>SHIRVAI</t>
@@ -3431,7 +3399,6 @@
           <t>Sulcorna</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
           <t>SURKARN</t>
@@ -3477,7 +3444,6 @@
           <t>Tiloi</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -3513,7 +3479,6 @@
           <t>Undorna</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
           <t>UDANA</t>
@@ -3619,7 +3584,6 @@
           <t>Xelvona</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
       <c r="L67" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -3655,7 +3619,6 @@
           <t>Xic-Xelvona</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
           <t>SHIKSHELVAN</t>
@@ -3706,7 +3669,6 @@
           <t>Zanodem</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
           <t>ZANODA</t>
@@ -3757,7 +3719,6 @@
           <t>Antoriem</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
           <t>ANTORIEM</t>
@@ -3803,7 +3764,6 @@
           <t>Bati</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
           <t>BATI</t>
@@ -3854,7 +3814,6 @@
           <t>Boma</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
           <t>BOMA</t>
@@ -3900,7 +3859,6 @@
           <t>Calem</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr">
         <is>
           <t>COLEM</t>
@@ -3946,7 +3904,6 @@
           <t>Colomb</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
           <t>KOLAMBA</t>
@@ -3997,7 +3954,6 @@
           <t>Comproi</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr">
         <is>
           <t>KANPRAY</t>
@@ -4043,7 +3999,6 @@
           <t>Coranginim</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr">
         <is>
           <t>KORANGUINIM</t>
@@ -4089,7 +4044,6 @@
           <t>Costi</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr">
         <is>
           <t>KASHTI</t>
@@ -4140,7 +4094,6 @@
           <t>Cotarli</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr">
         <is>
           <t>KOTARLI</t>
@@ -4186,7 +4139,6 @@
           <t>Cumbari</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
           <t>KUMBARI</t>
@@ -4232,7 +4184,6 @@
           <t>Curdem</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
           <t>KURDI</t>
@@ -4288,7 +4239,6 @@
           <t>Dongor</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
           <t>DONGAR</t>
@@ -4334,7 +4284,6 @@
           <t>Dongurli</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr">
         <is>
           <t>DONGURLI</t>
@@ -4380,7 +4329,6 @@
           <t>Dudal</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr">
         <is>
           <t>DUDAL</t>
@@ -4431,7 +4379,6 @@
           <t>Kurpem</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr">
         <is>
           <t>KURPE</t>
@@ -4482,7 +4429,6 @@
           <t>Maulinguem</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr">
         <is>
           <t>MALINGEM</t>
@@ -4528,7 +4474,6 @@
           <t>Muguli</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr">
         <is>
           <t>MUGULI</t>
@@ -4579,7 +4524,6 @@
           <t>Naiquinim</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr">
         <is>
           <t>NAIQUINIM</t>
@@ -4625,7 +4569,6 @@
           <t>Neturlim</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr">
         <is>
           <t>NETRAVLI</t>
@@ -4676,7 +4619,6 @@
           <t>Nundem</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr">
         <is>
           <t>NUNE</t>
@@ -4722,7 +4664,6 @@
           <t>Odxel</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr"/>
       <c r="F90" t="inlineStr">
         <is>
           <t>OXEL</t>
@@ -4768,7 +4709,6 @@
           <t>Patiem</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
           <t>PATIEM</t>
@@ -4814,7 +4754,6 @@
           <t>Porteem</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
           <t>PORTEM</t>
@@ -4860,7 +4799,6 @@
           <t>Potrem</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr">
         <is>
           <t>POTREM</t>
@@ -4906,7 +4844,6 @@
           <t>Rivona</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr">
         <is>
           <t>REVONA</t>
@@ -4962,7 +4899,6 @@
           <t>Rumbrem</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr">
         <is>
           <t>RUMBREM</t>
@@ -5013,7 +4949,6 @@
           <t>Salauli</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr">
         <is>
           <t>SALAVLI</t>
@@ -5059,7 +4994,6 @@
           <t>Sanguem</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr"/>
       <c r="L97" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -5095,7 +5029,6 @@
           <t>Santona</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr">
         <is>
           <t>SANTONA</t>
@@ -5196,7 +5129,6 @@
           <t>Sigonem</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr"/>
       <c r="F100" t="inlineStr">
         <is>
           <t>SIGONEM</t>
@@ -5247,7 +5179,6 @@
           <t>Todou</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr">
         <is>
           <t>TODOV</t>
@@ -5293,7 +5224,6 @@
           <t>Uguem</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr"/>
       <c r="F102" t="inlineStr">
         <is>
           <t>UGEM</t>
@@ -5344,7 +5274,6 @@
           <t>Verlem</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
       <c r="F103" t="inlineStr">
         <is>
           <t>VERLEN</t>
@@ -5395,7 +5324,6 @@
           <t>Vichundrem</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr"/>
       <c r="F104" t="inlineStr">
         <is>
           <t>DIGALI</t>
@@ -5446,7 +5374,6 @@
           <t>Viliena</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr">
         <is>
           <t>VILYAN</t>
@@ -5492,7 +5419,6 @@
           <t>Xelpem</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr">
         <is>
           <t>SHELPE</t>
@@ -5588,6 +5514,11 @@
       <c r="P107" s="2" t="n"/>
       <c r="Q107" s="2" t="n"/>
       <c r="R107" s="2" t="n"/>
+      <c r="V107" t="inlineStr">
+        <is>
+          <t>Oidone</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -5643,6 +5574,11 @@
       <c r="P108" s="2" t="n"/>
       <c r="Q108" s="2" t="n"/>
       <c r="R108" s="2" t="n"/>
+      <c r="V108" t="inlineStr">
+        <is>
+          <t>Honjunnem</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -5663,7 +5599,6 @@
           <t>Arpora</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr"/>
       <c r="F109" t="inlineStr">
         <is>
           <t>ARPORA</t>
@@ -5709,7 +5644,6 @@
           <t>Assagao</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
       <c r="F110" t="inlineStr">
         <is>
           <t>ASGAON</t>
@@ -5745,6 +5679,11 @@
       <c r="P110" s="2" t="n"/>
       <c r="Q110" s="2" t="n"/>
       <c r="R110" s="2" t="n"/>
+      <c r="V110" t="inlineStr">
+        <is>
+          <t>Fullyanchem Gaon</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -5765,7 +5704,6 @@
           <t>Assonora</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr">
         <is>
           <t>ASNODE</t>
@@ -5816,7 +5754,6 @@
           <t>Bastora</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
       <c r="L112" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -5892,6 +5829,11 @@
       <c r="P113" s="2" t="n"/>
       <c r="Q113" s="2" t="n"/>
       <c r="R113" s="2" t="n"/>
+      <c r="V113" t="inlineStr">
+        <is>
+          <t>Kolongutt</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -5912,7 +5854,6 @@
           <t>Calvim</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr"/>
       <c r="F114" t="inlineStr">
         <is>
           <t>KALVI</t>
@@ -5958,7 +5899,6 @@
           <t>Camurlim</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr"/>
       <c r="F115" t="inlineStr">
         <is>
           <t>OGALI</t>
@@ -6004,7 +5944,6 @@
           <t>Canca</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr"/>
       <c r="L116" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -6150,7 +6089,6 @@
           <t>Corjuem</t>
         </is>
       </c>
-      <c r="E119" t="inlineStr"/>
       <c r="F119" t="inlineStr">
         <is>
           <t>KHORUJUVEN</t>
@@ -6201,7 +6139,6 @@
           <t>Corlim</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr"/>
       <c r="L120" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -6237,7 +6174,6 @@
           <t>Cunchelim</t>
         </is>
       </c>
-      <c r="E121" t="inlineStr"/>
       <c r="L121" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -6333,7 +6269,6 @@
           <t>Marna</t>
         </is>
       </c>
-      <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr">
         <is>
           <t>SHIVOLI</t>
@@ -6384,7 +6319,6 @@
           <t>Marra</t>
         </is>
       </c>
-      <c r="E124" t="inlineStr"/>
       <c r="F124" t="inlineStr">
         <is>
           <t>MARRA</t>
@@ -6430,7 +6364,6 @@
           <t>Mhapsa</t>
         </is>
       </c>
-      <c r="E125" t="inlineStr"/>
       <c r="L125" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -6521,7 +6454,6 @@
           <t>Moitem</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr"/>
       <c r="F127" t="inlineStr">
         <is>
           <t>PIRNA</t>
@@ -6572,7 +6504,6 @@
           <t>Nachinola</t>
         </is>
       </c>
-      <c r="E128" t="inlineStr"/>
       <c r="F128" t="inlineStr">
         <is>
           <t>NACHINALA</t>
@@ -6618,7 +6549,6 @@
           <t>Nadora</t>
         </is>
       </c>
-      <c r="E129" t="inlineStr"/>
       <c r="F129" t="inlineStr">
         <is>
           <t>NEDORA</t>
@@ -6664,7 +6594,6 @@
           <t>Nagoa</t>
         </is>
       </c>
-      <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr">
         <is>
           <t>NAGVA</t>
@@ -6775,7 +6704,6 @@
           <t>Olaulim</t>
         </is>
       </c>
-      <c r="E132" t="inlineStr"/>
       <c r="F132" t="inlineStr">
         <is>
           <t>VOLAWALI</t>
@@ -6821,7 +6749,6 @@
           <t>Oxel</t>
         </is>
       </c>
-      <c r="E133" t="inlineStr"/>
       <c r="F133" t="inlineStr">
         <is>
           <t>OSHAL</t>
@@ -6872,7 +6799,6 @@
           <t>Paliem</t>
         </is>
       </c>
-      <c r="E134" t="inlineStr"/>
       <c r="F134" t="inlineStr">
         <is>
           <t>PALIYE</t>
@@ -6918,7 +6844,6 @@
           <t>Parra</t>
         </is>
       </c>
-      <c r="E135" t="inlineStr"/>
       <c r="F135" t="inlineStr">
         <is>
           <t>PARRA</t>
@@ -7074,7 +6999,6 @@
           <t>Pirna</t>
         </is>
       </c>
-      <c r="E138" t="inlineStr"/>
       <c r="L138" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -7110,7 +7034,6 @@
           <t>Pomburpa</t>
         </is>
       </c>
-      <c r="E139" t="inlineStr"/>
       <c r="F139" t="inlineStr">
         <is>
           <t>POMBURPA</t>
@@ -7161,7 +7084,6 @@
           <t>Ponolem</t>
         </is>
       </c>
-      <c r="E140" t="inlineStr"/>
       <c r="L140" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -7197,7 +7119,6 @@
           <t>Punola</t>
         </is>
       </c>
-      <c r="E141" t="inlineStr"/>
       <c r="L141" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -7233,7 +7154,6 @@
           <t>Reis-Magos</t>
         </is>
       </c>
-      <c r="E142" t="inlineStr"/>
       <c r="L142" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -7269,7 +7189,6 @@
           <t>Revora</t>
         </is>
       </c>
-      <c r="E143" t="inlineStr"/>
       <c r="L143" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -7415,7 +7334,6 @@
           <t>Sangolda</t>
         </is>
       </c>
-      <c r="E146" t="inlineStr"/>
       <c r="F146" t="inlineStr">
         <is>
           <t>SANGOLDA</t>
@@ -7521,7 +7439,6 @@
           <t>Sircaim</t>
         </is>
       </c>
-      <c r="E148" t="inlineStr"/>
       <c r="F148" t="inlineStr">
         <is>
           <t>SIRSAI</t>
@@ -7627,7 +7544,6 @@
           <t>Tivim</t>
         </is>
       </c>
-      <c r="E150" t="inlineStr"/>
       <c r="F150" t="inlineStr">
         <is>
           <t>DAT</t>
@@ -7678,7 +7594,6 @@
           <t>Ucassaim</t>
         </is>
       </c>
-      <c r="E151" t="inlineStr"/>
       <c r="F151" t="inlineStr">
         <is>
           <t>UKSAI</t>
@@ -7724,7 +7639,6 @@
           <t>Verla</t>
         </is>
       </c>
-      <c r="E152" t="inlineStr"/>
       <c r="F152" t="inlineStr">
         <is>
           <t>PARRA</t>
@@ -7775,7 +7689,6 @@
           <t>Adwalpale</t>
         </is>
       </c>
-      <c r="E153" t="inlineStr"/>
       <c r="F153" t="inlineStr">
         <is>
           <t>ADVALPAL</t>
@@ -7826,7 +7739,6 @@
           <t>Amone</t>
         </is>
       </c>
-      <c r="E154" t="inlineStr"/>
       <c r="F154" t="inlineStr">
         <is>
           <t>AMONA</t>
@@ -7872,7 +7784,6 @@
           <t>Arvalem</t>
         </is>
       </c>
-      <c r="E155" t="inlineStr"/>
       <c r="L155" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -7908,7 +7819,6 @@
           <t>Aturli</t>
         </is>
       </c>
-      <c r="E156" t="inlineStr"/>
       <c r="F156" t="inlineStr">
         <is>
           <t>ATURLI</t>
@@ -7959,7 +7869,6 @@
           <t>Bicholim</t>
         </is>
       </c>
-      <c r="E157" t="inlineStr"/>
       <c r="L157" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -7975,6 +7884,11 @@
       <c r="P157" s="2" t="n"/>
       <c r="Q157" s="2" t="n"/>
       <c r="R157" s="2" t="n"/>
+      <c r="V157" t="inlineStr">
+        <is>
+          <t>Divchali</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -7995,7 +7909,6 @@
           <t>Bordem</t>
         </is>
       </c>
-      <c r="E158" t="inlineStr"/>
       <c r="L158" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -8086,7 +7999,6 @@
           <t>Cotombi</t>
         </is>
       </c>
-      <c r="E160" t="inlineStr"/>
       <c r="F160" t="inlineStr">
         <is>
           <t>KOTAMBI</t>
@@ -8132,7 +8044,6 @@
           <t>Cudnem</t>
         </is>
       </c>
-      <c r="E161" t="inlineStr"/>
       <c r="F161" t="inlineStr">
         <is>
           <t>KUDNE</t>
@@ -8183,7 +8094,6 @@
           <t>Curchirem</t>
         </is>
       </c>
-      <c r="E162" t="inlineStr"/>
       <c r="F162" t="inlineStr">
         <is>
           <t>KUDCHIRE</t>
@@ -8229,7 +8139,6 @@
           <t>Dumacem</t>
         </is>
       </c>
-      <c r="E163" t="inlineStr"/>
       <c r="F163" t="inlineStr">
         <is>
           <t>DUMASE</t>
@@ -8280,7 +8189,6 @@
           <t>Lamgao</t>
         </is>
       </c>
-      <c r="E164" t="inlineStr"/>
       <c r="L164" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -8316,7 +8224,6 @@
           <t>Latambarcem</t>
         </is>
       </c>
-      <c r="E165" t="inlineStr"/>
       <c r="F165" t="inlineStr">
         <is>
           <t>KASARPAL</t>
@@ -8362,7 +8269,6 @@
           <t>Maem</t>
         </is>
       </c>
-      <c r="E166" t="inlineStr"/>
       <c r="F166" t="inlineStr">
         <is>
           <t>BHATWADI</t>
@@ -8393,6 +8299,11 @@
       <c r="P166" s="2" t="n"/>
       <c r="Q166" s="2" t="n"/>
       <c r="R166" s="2" t="n"/>
+      <c r="V166" t="inlineStr">
+        <is>
+          <t>Mayem</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -8413,7 +8324,6 @@
           <t>Maulinguem South</t>
         </is>
       </c>
-      <c r="E167" t="inlineStr"/>
       <c r="L167" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -8449,7 +8359,6 @@
           <t>Maulinguem-North</t>
         </is>
       </c>
-      <c r="E168" t="inlineStr"/>
       <c r="F168" t="inlineStr">
         <is>
           <t>MAVLINGE</t>
@@ -8495,7 +8404,6 @@
           <t>Mencurem</t>
         </is>
       </c>
-      <c r="E169" t="inlineStr"/>
       <c r="F169" t="inlineStr">
         <is>
           <t>MENKURE</t>
@@ -8541,7 +8449,6 @@
           <t>Mulgao</t>
         </is>
       </c>
-      <c r="E170" t="inlineStr"/>
       <c r="F170" t="inlineStr">
         <is>
           <t>MULGAON</t>
@@ -8587,13 +8494,11 @@
           <t>Naroa</t>
         </is>
       </c>
-      <c r="E171" t="inlineStr"/>
       <c r="F171" t="inlineStr">
         <is>
           <t>NARVA</t>
         </is>
       </c>
-      <c r="G171" t="inlineStr"/>
       <c r="J171" t="inlineStr">
         <is>
           <t>नार्वें</t>
@@ -8634,7 +8539,6 @@
           <t>Navelim</t>
         </is>
       </c>
-      <c r="E172" t="inlineStr"/>
       <c r="F172" t="inlineStr">
         <is>
           <t>BHARINBAG</t>
@@ -8685,7 +8589,6 @@
           <t>Ona</t>
         </is>
       </c>
-      <c r="E173" t="inlineStr"/>
       <c r="F173" t="inlineStr">
         <is>
           <t>ON</t>
@@ -8796,7 +8699,6 @@
           <t>Piligao</t>
         </is>
       </c>
-      <c r="E175" t="inlineStr"/>
       <c r="F175" t="inlineStr">
         <is>
           <t>PILIGAON</t>
@@ -8842,7 +8744,6 @@
           <t>Salem</t>
         </is>
       </c>
-      <c r="E176" t="inlineStr"/>
       <c r="F176" t="inlineStr">
         <is>
           <t>SAL</t>
@@ -8888,7 +8789,6 @@
           <t>Sankhali</t>
         </is>
       </c>
-      <c r="E177" t="inlineStr"/>
       <c r="L177" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -8924,7 +8824,6 @@
           <t>Sarvona</t>
         </is>
       </c>
-      <c r="E178" t="inlineStr"/>
       <c r="F178" t="inlineStr">
         <is>
           <t>SARVAN</t>
@@ -8975,7 +8874,6 @@
           <t>Sirigao</t>
         </is>
       </c>
-      <c r="E179" t="inlineStr"/>
       <c r="L179" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -9011,7 +8909,6 @@
           <t>Surla</t>
         </is>
       </c>
-      <c r="E180" t="inlineStr"/>
       <c r="F180" t="inlineStr">
         <is>
           <t>DINGNASUR</t>
@@ -9057,7 +8954,6 @@
           <t>Vainguinim</t>
         </is>
       </c>
-      <c r="E181" t="inlineStr"/>
       <c r="F181" t="inlineStr">
         <is>
           <t>VAYANGNE</t>
@@ -9103,7 +8999,6 @@
           <t>Velguem</t>
         </is>
       </c>
-      <c r="E182" t="inlineStr"/>
       <c r="F182" t="inlineStr">
         <is>
           <t>VELGE</t>
@@ -9154,7 +9049,6 @@
           <t>Virdi</t>
         </is>
       </c>
-      <c r="E183" t="inlineStr"/>
       <c r="L183" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -9190,7 +9084,6 @@
           <t>Agarvado</t>
         </is>
       </c>
-      <c r="E184" t="inlineStr"/>
       <c r="F184" t="inlineStr">
         <is>
           <t>AGARVADA</t>
@@ -9241,7 +9134,6 @@
           <t>Alorna</t>
         </is>
       </c>
-      <c r="E185" t="inlineStr"/>
       <c r="F185" t="inlineStr">
         <is>
           <t>ALORNA</t>
@@ -9287,7 +9179,6 @@
           <t>Amberem</t>
         </is>
       </c>
-      <c r="E186" t="inlineStr"/>
       <c r="L186" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -9378,7 +9269,6 @@
           <t>Cansarvornem</t>
         </is>
       </c>
-      <c r="E188" t="inlineStr"/>
       <c r="F188" t="inlineStr">
         <is>
           <t>KASARVARNE</t>
@@ -9429,7 +9319,6 @@
           <t>Casnem</t>
         </is>
       </c>
-      <c r="E189" t="inlineStr"/>
       <c r="L189" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -9465,7 +9354,6 @@
           <t>Chandel</t>
         </is>
       </c>
-      <c r="E190" t="inlineStr"/>
       <c r="F190" t="inlineStr">
         <is>
           <t>CHANDEL</t>
@@ -9511,7 +9399,6 @@
           <t>Chopdem</t>
         </is>
       </c>
-      <c r="E191" t="inlineStr"/>
       <c r="L191" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -9547,7 +9434,6 @@
           <t>Corgao</t>
         </is>
       </c>
-      <c r="E192" t="inlineStr"/>
       <c r="F192" t="inlineStr">
         <is>
           <t>KORGAON</t>
@@ -9593,7 +9479,6 @@
           <t>Dargalim</t>
         </is>
       </c>
-      <c r="E193" t="inlineStr"/>
       <c r="F193" t="inlineStr">
         <is>
           <t>DHARGAL</t>
@@ -9644,7 +9529,6 @@
           <t>Ibrampur</t>
         </is>
       </c>
-      <c r="E194" t="inlineStr"/>
       <c r="F194" t="inlineStr">
         <is>
           <t>IBRAMPUR</t>
@@ -9735,6 +9619,11 @@
       <c r="P195" s="2" t="n"/>
       <c r="Q195" s="2" t="n"/>
       <c r="R195" s="2" t="n"/>
+      <c r="V195" t="inlineStr">
+        <is>
+          <t>Mandre</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -9755,7 +9644,6 @@
           <t>Mopa</t>
         </is>
       </c>
-      <c r="E196" t="inlineStr"/>
       <c r="F196" t="inlineStr">
         <is>
           <t>MOPA</t>
@@ -9811,7 +9699,6 @@
           <t>Morgim</t>
         </is>
       </c>
-      <c r="E197" t="inlineStr"/>
       <c r="F197" t="inlineStr">
         <is>
           <t>MORJIM</t>
@@ -9867,7 +9754,6 @@
           <t>Ozorim</t>
         </is>
       </c>
-      <c r="E198" t="inlineStr"/>
       <c r="F198" t="inlineStr">
         <is>
           <t>VAJRI</t>
@@ -9913,7 +9799,6 @@
           <t>Paliem</t>
         </is>
       </c>
-      <c r="E199" t="inlineStr"/>
       <c r="F199" t="inlineStr">
         <is>
           <t>PALIEM</t>
@@ -10019,7 +9904,6 @@
           <t>Pernem</t>
         </is>
       </c>
-      <c r="E201" t="inlineStr"/>
       <c r="L201" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -10055,7 +9939,6 @@
           <t>Poroscodem</t>
         </is>
       </c>
-      <c r="E202" t="inlineStr"/>
       <c r="F202" t="inlineStr">
         <is>
           <t>PARASKAD</t>
@@ -10101,7 +9984,6 @@
           <t>Querim</t>
         </is>
       </c>
-      <c r="E203" t="inlineStr"/>
       <c r="F203" t="inlineStr">
         <is>
           <t>QUERIM</t>
@@ -10147,7 +10029,6 @@
           <t>Tamboxem</t>
         </is>
       </c>
-      <c r="E204" t="inlineStr"/>
       <c r="F204" t="inlineStr">
         <is>
           <t>TAMBOSE</t>
@@ -10198,7 +10079,6 @@
           <t>Tiracol</t>
         </is>
       </c>
-      <c r="E205" t="inlineStr"/>
       <c r="F205" t="inlineStr">
         <is>
           <t>TIRACOL</t>
@@ -10244,7 +10124,6 @@
           <t>Torxem</t>
         </is>
       </c>
-      <c r="E206" t="inlineStr"/>
       <c r="F206" t="inlineStr">
         <is>
           <t>TORSE</t>
@@ -10290,7 +10169,6 @@
           <t>Tuem</t>
         </is>
       </c>
-      <c r="E207" t="inlineStr"/>
       <c r="F207" t="inlineStr">
         <is>
           <t>TUYE</t>
@@ -10336,7 +10214,6 @@
           <t>Uguem</t>
         </is>
       </c>
-      <c r="E208" t="inlineStr"/>
       <c r="F208" t="inlineStr">
         <is>
           <t>UGUEM</t>
@@ -10382,7 +10259,6 @@
           <t>Varconda</t>
         </is>
       </c>
-      <c r="E209" t="inlineStr"/>
       <c r="F209" t="inlineStr">
         <is>
           <t>VARKHAND</t>
@@ -10428,7 +10304,6 @@
           <t>Virnora</t>
         </is>
       </c>
-      <c r="E210" t="inlineStr"/>
       <c r="F210" t="inlineStr">
         <is>
           <t>VIRNODA</t>
@@ -10479,7 +10354,6 @@
           <t>Advoi</t>
         </is>
       </c>
-      <c r="E211" t="inlineStr"/>
       <c r="F211" t="inlineStr">
         <is>
           <t>ADVAI DESAIWADA</t>
@@ -10525,7 +10399,6 @@
           <t>Ambedem</t>
         </is>
       </c>
-      <c r="E212" t="inlineStr"/>
       <c r="F212" t="inlineStr">
         <is>
           <t>AMBEDE</t>
@@ -10576,7 +10449,6 @@
           <t>Ambeli</t>
         </is>
       </c>
-      <c r="E213" t="inlineStr"/>
       <c r="F213" t="inlineStr">
         <is>
           <t>AMBELI</t>
@@ -10627,7 +10499,6 @@
           <t>Anjunem</t>
         </is>
       </c>
-      <c r="E214" t="inlineStr"/>
       <c r="F214" t="inlineStr">
         <is>
           <t>ANJUNE</t>
@@ -10673,7 +10544,6 @@
           <t>Ansolem</t>
         </is>
       </c>
-      <c r="E215" t="inlineStr"/>
       <c r="L215" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -10709,7 +10579,6 @@
           <t>Assodem</t>
         </is>
       </c>
-      <c r="E216" t="inlineStr"/>
       <c r="F216" t="inlineStr">
         <is>
           <t>AASSODE</t>
@@ -10760,7 +10629,6 @@
           <t>Birondem</t>
         </is>
       </c>
-      <c r="E217" t="inlineStr"/>
       <c r="F217" t="inlineStr">
         <is>
           <t>BHIRONDE</t>
@@ -10806,7 +10674,6 @@
           <t>Bombedem</t>
         </is>
       </c>
-      <c r="E218" t="inlineStr"/>
       <c r="F218" t="inlineStr">
         <is>
           <t>BOMBEDE</t>
@@ -10857,7 +10724,6 @@
           <t>Buimpal</t>
         </is>
       </c>
-      <c r="E219" t="inlineStr"/>
       <c r="F219" t="inlineStr">
         <is>
           <t>BHUIPAL</t>
@@ -10908,7 +10774,6 @@
           <t>Carambolim- Brama</t>
         </is>
       </c>
-      <c r="E220" t="inlineStr"/>
       <c r="F220" t="inlineStr">
         <is>
           <t>KARAMBALI BRAMHA</t>
@@ -10954,7 +10819,6 @@
           <t>Carambolim-Buzruco</t>
         </is>
       </c>
-      <c r="E221" t="inlineStr"/>
       <c r="F221" t="inlineStr">
         <is>
           <t>KARAMBALI BUZRUK</t>
@@ -11005,7 +10869,6 @@
           <t>Caranzol</t>
         </is>
       </c>
-      <c r="E222" t="inlineStr"/>
       <c r="F222" t="inlineStr">
         <is>
           <t>KARANZOL</t>
@@ -11051,7 +10914,6 @@
           <t>Choraundem</t>
         </is>
       </c>
-      <c r="E223" t="inlineStr"/>
       <c r="F223" t="inlineStr">
         <is>
           <t>CHARAVADE</t>
@@ -11097,7 +10959,6 @@
           <t>Codal</t>
         </is>
       </c>
-      <c r="E224" t="inlineStr"/>
       <c r="F224" t="inlineStr">
         <is>
           <t>KODAL</t>
@@ -11143,7 +11004,6 @@
           <t>Codiem</t>
         </is>
       </c>
-      <c r="E225" t="inlineStr"/>
       <c r="F225" t="inlineStr">
         <is>
           <t>HASOLE</t>
@@ -11189,7 +11049,6 @@
           <t>Codqui</t>
         </is>
       </c>
-      <c r="E226" t="inlineStr"/>
       <c r="F226" t="inlineStr">
         <is>
           <t>BARAJAN</t>
@@ -11235,7 +11094,6 @@
           <t>Codvol</t>
         </is>
       </c>
-      <c r="E227" t="inlineStr"/>
       <c r="F227" t="inlineStr">
         <is>
           <t>KODAL</t>
@@ -11286,7 +11144,6 @@
           <t>Compordem</t>
         </is>
       </c>
-      <c r="E228" t="inlineStr"/>
       <c r="L228" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -11322,7 +11179,6 @@
           <t>Conquirem</t>
         </is>
       </c>
-      <c r="E229" t="inlineStr"/>
       <c r="L229" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -11358,7 +11214,6 @@
           <t>Cotorem</t>
         </is>
       </c>
-      <c r="E230" t="inlineStr"/>
       <c r="F230" t="inlineStr">
         <is>
           <t>KHOTODE</t>
@@ -11409,7 +11264,6 @@
           <t>Cudcem</t>
         </is>
       </c>
-      <c r="E231" t="inlineStr"/>
       <c r="L231" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -11445,7 +11299,6 @@
           <t>Cumarconda</t>
         </is>
       </c>
-      <c r="E232" t="inlineStr"/>
       <c r="F232" t="inlineStr">
         <is>
           <t>KUMAR KHAND</t>
@@ -11496,7 +11349,6 @@
           <t>Dabem</t>
         </is>
       </c>
-      <c r="E233" t="inlineStr"/>
       <c r="L233" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -11532,7 +11384,6 @@
           <t>Damocem</t>
         </is>
       </c>
-      <c r="E234" t="inlineStr"/>
       <c r="F234" t="inlineStr">
         <is>
           <t>DHAMSE</t>
@@ -11583,7 +11434,6 @@
           <t>Davem</t>
         </is>
       </c>
-      <c r="E235" t="inlineStr"/>
       <c r="F235" t="inlineStr">
         <is>
           <t>DONGARVADA</t>
@@ -11634,7 +11484,6 @@
           <t>Derodem</t>
         </is>
       </c>
-      <c r="E236" t="inlineStr"/>
       <c r="F236" t="inlineStr">
         <is>
           <t>DERODE</t>
@@ -11685,7 +11534,6 @@
           <t>Dongurli</t>
         </is>
       </c>
-      <c r="E237" t="inlineStr"/>
       <c r="F237" t="inlineStr">
         <is>
           <t>DONGURVADA</t>
@@ -11736,7 +11584,6 @@
           <t>Edorem</t>
         </is>
       </c>
-      <c r="E238" t="inlineStr"/>
       <c r="F238" t="inlineStr">
         <is>
           <t>KOPARDE</t>
@@ -11787,7 +11634,6 @@
           <t>Golauli</t>
         </is>
       </c>
-      <c r="E239" t="inlineStr"/>
       <c r="F239" t="inlineStr">
         <is>
           <t>GOALI</t>
@@ -11833,7 +11679,6 @@
           <t>Gonteli</t>
         </is>
       </c>
-      <c r="E240" t="inlineStr"/>
       <c r="F240" t="inlineStr">
         <is>
           <t>GHONTELI</t>
@@ -11884,7 +11729,6 @@
           <t>Govanem</t>
         </is>
       </c>
-      <c r="E241" t="inlineStr"/>
       <c r="F241" t="inlineStr">
         <is>
           <t>GAVANE</t>
@@ -11935,7 +11779,6 @@
           <t>Guleli</t>
         </is>
       </c>
-      <c r="E242" t="inlineStr"/>
       <c r="F242" t="inlineStr">
         <is>
           <t>GULELI</t>
@@ -11986,7 +11829,6 @@
           <t>Gululem</t>
         </is>
       </c>
-      <c r="E243" t="inlineStr"/>
       <c r="F243" t="inlineStr">
         <is>
           <t>GULLE</t>
@@ -12032,7 +11874,6 @@
           <t>Ivrem-Buzruco</t>
         </is>
       </c>
-      <c r="E244" t="inlineStr"/>
       <c r="F244" t="inlineStr">
         <is>
           <t>IVRE BUDRUK</t>
@@ -12083,7 +11924,6 @@
           <t>Ivrem-Curdo</t>
         </is>
       </c>
-      <c r="E245" t="inlineStr"/>
       <c r="F245" t="inlineStr">
         <is>
           <t>IVRE KHURD</t>
@@ -12129,7 +11969,6 @@
           <t>Maloli</t>
         </is>
       </c>
-      <c r="E246" t="inlineStr"/>
       <c r="F246" t="inlineStr">
         <is>
           <t>MALOLI</t>
@@ -12180,7 +12019,6 @@
           <t>Malpona</t>
         </is>
       </c>
-      <c r="E247" t="inlineStr"/>
       <c r="F247" t="inlineStr">
         <is>
           <t>MALPON</t>
@@ -12226,7 +12064,6 @@
           <t>Massordem</t>
         </is>
       </c>
-      <c r="E248" t="inlineStr"/>
       <c r="L248" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -12262,7 +12099,6 @@
           <t>Mauxi</t>
         </is>
       </c>
-      <c r="E249" t="inlineStr"/>
       <c r="F249" t="inlineStr">
         <is>
           <t>MAUSI</t>
@@ -12308,7 +12144,6 @@
           <t>Melauli</t>
         </is>
       </c>
-      <c r="E250" t="inlineStr"/>
       <c r="F250" t="inlineStr">
         <is>
           <t>MELAVALI</t>
@@ -12359,7 +12194,6 @@
           <t>Morlem</t>
         </is>
       </c>
-      <c r="E251" t="inlineStr"/>
       <c r="F251" t="inlineStr">
         <is>
           <t>MORLE</t>
@@ -12410,7 +12244,6 @@
           <t>Nagargao</t>
         </is>
       </c>
-      <c r="E252" t="inlineStr"/>
       <c r="L252" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -12446,7 +12279,6 @@
           <t>Naguem</t>
         </is>
       </c>
-      <c r="E253" t="inlineStr"/>
       <c r="F253" t="inlineStr">
         <is>
           <t>Naguem</t>
@@ -12492,7 +12324,6 @@
           <t>Naneli</t>
         </is>
       </c>
-      <c r="E254" t="inlineStr"/>
       <c r="F254" t="inlineStr">
         <is>
           <t>NANELI</t>
@@ -12543,7 +12374,6 @@
           <t>Nanorem</t>
         </is>
       </c>
-      <c r="E255" t="inlineStr"/>
       <c r="F255" t="inlineStr">
         <is>
           <t>NANODE</t>
@@ -12589,7 +12419,6 @@
           <t>Nanus</t>
         </is>
       </c>
-      <c r="E256" t="inlineStr"/>
       <c r="L256" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -12680,7 +12509,6 @@
           <t>Padeli</t>
         </is>
       </c>
-      <c r="E258" t="inlineStr"/>
       <c r="F258" t="inlineStr">
         <is>
           <t>BHOMWADI</t>
@@ -12726,7 +12554,6 @@
           <t>Pale</t>
         </is>
       </c>
-      <c r="E259" t="inlineStr"/>
       <c r="F259" t="inlineStr">
         <is>
           <t>PALI</t>
@@ -12777,7 +12604,6 @@
           <t>Pendral</t>
         </is>
       </c>
-      <c r="E260" t="inlineStr"/>
       <c r="F260" t="inlineStr">
         <is>
           <t>PENRAL</t>
@@ -12823,7 +12649,6 @@
           <t>Pissurlem</t>
         </is>
       </c>
-      <c r="E261" t="inlineStr"/>
       <c r="F261" t="inlineStr">
         <is>
           <t>PISSURLE</t>
@@ -12874,7 +12699,6 @@
           <t>Podocem</t>
         </is>
       </c>
-      <c r="E262" t="inlineStr"/>
       <c r="F262" t="inlineStr">
         <is>
           <t>PODSEN</t>
@@ -12920,7 +12744,6 @@
           <t>Ponocem</t>
         </is>
       </c>
-      <c r="E263" t="inlineStr"/>
       <c r="F263" t="inlineStr">
         <is>
           <t>PANSE</t>
@@ -12966,7 +12789,6 @@
           <t>Ponsuli</t>
         </is>
       </c>
-      <c r="E264" t="inlineStr"/>
       <c r="L264" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -13002,7 +12824,6 @@
           <t>Poriem</t>
         </is>
       </c>
-      <c r="E265" t="inlineStr"/>
       <c r="F265" t="inlineStr">
         <is>
           <t>PARIYE</t>
@@ -13048,7 +12869,6 @@
           <t>Quelaudem</t>
         </is>
       </c>
-      <c r="E266" t="inlineStr"/>
       <c r="F266" t="inlineStr">
         <is>
           <t>KELAVADE</t>
@@ -13094,7 +12914,6 @@
           <t>Querim</t>
         </is>
       </c>
-      <c r="E267" t="inlineStr"/>
       <c r="F267" t="inlineStr">
         <is>
           <t>BAYALVADA</t>
@@ -13140,7 +12959,6 @@
           <t>Ravona</t>
         </is>
       </c>
-      <c r="E268" t="inlineStr"/>
       <c r="F268" t="inlineStr">
         <is>
           <t>RAVAN</t>
@@ -13186,7 +13004,6 @@
           <t>Rivem</t>
         </is>
       </c>
-      <c r="E269" t="inlineStr"/>
       <c r="F269" t="inlineStr">
         <is>
           <t>RIVE</t>
@@ -13232,7 +13049,6 @@
           <t>Saleli</t>
         </is>
       </c>
-      <c r="E270" t="inlineStr"/>
       <c r="F270" t="inlineStr">
         <is>
           <t>SALILI</t>
@@ -13278,7 +13094,6 @@
           <t>Sanvorcem</t>
         </is>
       </c>
-      <c r="E271" t="inlineStr"/>
       <c r="F271" t="inlineStr">
         <is>
           <t>SANVARSHE</t>
@@ -13324,7 +13139,6 @@
           <t>Sanvordem</t>
         </is>
       </c>
-      <c r="E272" t="inlineStr"/>
       <c r="F272" t="inlineStr">
         <is>
           <t>SANVARDE</t>
@@ -13375,7 +13189,6 @@
           <t>Satorem</t>
         </is>
       </c>
-      <c r="E273" t="inlineStr"/>
       <c r="F273" t="inlineStr">
         <is>
           <t>HEDODE</t>
@@ -13426,7 +13239,6 @@
           <t>Satrem</t>
         </is>
       </c>
-      <c r="E274" t="inlineStr"/>
       <c r="F274" t="inlineStr">
         <is>
           <t>SATRE</t>
@@ -13472,7 +13284,6 @@
           <t>Sigonem</t>
         </is>
       </c>
-      <c r="E275" t="inlineStr"/>
       <c r="F275" t="inlineStr">
         <is>
           <t>SINGNA</t>
@@ -13518,7 +13329,6 @@
           <t>Siranguli</t>
         </is>
       </c>
-      <c r="E276" t="inlineStr"/>
       <c r="L276" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -13554,7 +13364,6 @@
           <t>Siroli</t>
         </is>
       </c>
-      <c r="E277" t="inlineStr"/>
       <c r="F277" t="inlineStr">
         <is>
           <t>SHIROLI</t>
@@ -13605,7 +13414,6 @@
           <t>Sirsodem</t>
         </is>
       </c>
-      <c r="E278" t="inlineStr"/>
       <c r="F278" t="inlineStr">
         <is>
           <t>SIRSODE</t>
@@ -13651,7 +13459,6 @@
           <t>Sonal</t>
         </is>
       </c>
-      <c r="E279" t="inlineStr"/>
       <c r="F279" t="inlineStr">
         <is>
           <t>SONAL</t>
@@ -13697,7 +13504,6 @@
           <t>Sonus-Vonvoliem</t>
         </is>
       </c>
-      <c r="E280" t="inlineStr"/>
       <c r="F280" t="inlineStr">
         <is>
           <t>OVALAYEN</t>
@@ -13743,7 +13549,6 @@
           <t>Surla</t>
         </is>
       </c>
-      <c r="E281" t="inlineStr"/>
       <c r="F281" t="inlineStr">
         <is>
           <t>SURLA</t>
@@ -13789,7 +13594,6 @@
           <t>Ustem</t>
         </is>
       </c>
-      <c r="E282" t="inlineStr"/>
       <c r="F282" t="inlineStr">
         <is>
           <t>USTE</t>
@@ -13840,7 +13644,6 @@
           <t>Vaguriem</t>
         </is>
       </c>
-      <c r="E283" t="inlineStr"/>
       <c r="F283" t="inlineStr">
         <is>
           <t>WAGURE</t>
@@ -13886,7 +13689,6 @@
           <t>Vainguinim</t>
         </is>
       </c>
-      <c r="E284" t="inlineStr"/>
       <c r="F284" t="inlineStr">
         <is>
           <t>VAYANGANI</t>
@@ -13932,7 +13734,6 @@
           <t>Valpoi</t>
         </is>
       </c>
-      <c r="E285" t="inlineStr"/>
       <c r="L285" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -13968,7 +13769,6 @@
           <t>Vantem</t>
         </is>
       </c>
-      <c r="E286" t="inlineStr"/>
       <c r="F286" t="inlineStr">
         <is>
           <t>VANTE GAONKARWADA</t>
@@ -14014,7 +13814,6 @@
           <t>Velguem</t>
         </is>
       </c>
-      <c r="E287" t="inlineStr"/>
       <c r="F287" t="inlineStr">
         <is>
           <t>VELGUE</t>
@@ -14060,7 +13859,6 @@
           <t>Velus</t>
         </is>
       </c>
-      <c r="E288" t="inlineStr"/>
       <c r="L288" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -14096,7 +13894,6 @@
           <t>Xelopo-Buzruco</t>
         </is>
       </c>
-      <c r="E289" t="inlineStr"/>
       <c r="F289" t="inlineStr">
         <is>
           <t>SALPI BUDRUK</t>
@@ -14142,7 +13939,6 @@
           <t>Xelopo-Curdo</t>
         </is>
       </c>
-      <c r="E290" t="inlineStr"/>
       <c r="F290" t="inlineStr">
         <is>
           <t>SHELPI KHURD</t>
@@ -14193,7 +13989,6 @@
           <t>Zarani</t>
         </is>
       </c>
-      <c r="E291" t="inlineStr"/>
       <c r="L291" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -14229,7 +14024,6 @@
           <t>Zormen</t>
         </is>
       </c>
-      <c r="E292" t="inlineStr"/>
       <c r="F292" t="inlineStr">
         <is>
           <t>JARMA</t>
@@ -14275,7 +14069,6 @@
           <t>Ambarim</t>
         </is>
       </c>
-      <c r="E293" t="inlineStr"/>
       <c r="L293" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -14311,7 +14104,6 @@
           <t>Azossim</t>
         </is>
       </c>
-      <c r="E294" t="inlineStr"/>
       <c r="F294" t="inlineStr">
         <is>
           <t>AJOSI</t>
@@ -14357,7 +14149,6 @@
           <t>Bainguinim</t>
         </is>
       </c>
-      <c r="E295" t="inlineStr"/>
       <c r="F295" t="inlineStr">
         <is>
           <t>BAINGINI</t>
@@ -14463,7 +14254,6 @@
           <t>Batim</t>
         </is>
       </c>
-      <c r="E297" t="inlineStr"/>
       <c r="L297" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -14554,7 +14344,6 @@
           <t>Capao</t>
         </is>
       </c>
-      <c r="E299" t="inlineStr"/>
       <c r="F299" t="inlineStr">
         <is>
           <t>VANSHI</t>
@@ -14600,7 +14389,6 @@
           <t>Caraim</t>
         </is>
       </c>
-      <c r="E300" t="inlineStr"/>
       <c r="F300" t="inlineStr">
         <is>
           <t>MADEL</t>
@@ -14646,7 +14434,6 @@
           <t>Carambolim</t>
         </is>
       </c>
-      <c r="E301" t="inlineStr"/>
       <c r="F301" t="inlineStr">
         <is>
           <t>KARMALI</t>
@@ -14752,7 +14539,6 @@
           <t>Chorao</t>
         </is>
       </c>
-      <c r="E303" t="inlineStr"/>
       <c r="L303" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -14768,6 +14554,11 @@
       <c r="P303" s="2" t="n"/>
       <c r="Q303" s="2" t="n"/>
       <c r="R303" s="2" t="n"/>
+      <c r="V303" t="inlineStr">
+        <is>
+          <t>Choddnnem</t>
+        </is>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="n">
@@ -14948,7 +14739,6 @@
           <t>Curca</t>
         </is>
       </c>
-      <c r="E307" t="inlineStr"/>
       <c r="F307" t="inlineStr">
         <is>
           <t>KURKA</t>
@@ -14994,7 +14784,6 @@
           <t>Durgavado</t>
         </is>
       </c>
-      <c r="E308" t="inlineStr"/>
       <c r="L308" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -15030,7 +14819,6 @@
           <t>Ella</t>
         </is>
       </c>
-      <c r="E309" t="inlineStr"/>
       <c r="F309" t="inlineStr">
         <is>
           <t>VELA</t>
@@ -15081,7 +14869,6 @@
           <t>Gancim</t>
         </is>
       </c>
-      <c r="E310" t="inlineStr"/>
       <c r="F310" t="inlineStr">
         <is>
           <t>GANSIM</t>
@@ -15127,7 +14914,6 @@
           <t>Gandaulim</t>
         </is>
       </c>
-      <c r="E311" t="inlineStr"/>
       <c r="L311" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -15143,6 +14929,11 @@
       <c r="P311" s="2" t="n"/>
       <c r="Q311" s="2" t="n"/>
       <c r="R311" s="2" t="n"/>
+      <c r="V311" t="inlineStr">
+        <is>
+          <t>Gaundale</t>
+        </is>
+      </c>
     </row>
     <row r="312">
       <c r="A312" t="n">
@@ -15163,7 +14954,6 @@
           <t>Goa-Velha</t>
         </is>
       </c>
-      <c r="E312" t="inlineStr"/>
       <c r="F312" t="inlineStr">
         <is>
           <t>GOA VELHA</t>
@@ -15194,6 +14984,11 @@
       <c r="P312" s="2" t="n"/>
       <c r="Q312" s="2" t="n"/>
       <c r="R312" s="2" t="n"/>
+      <c r="V312" t="inlineStr">
+        <is>
+          <t>Vhoddlem Goem</t>
+        </is>
+      </c>
     </row>
     <row r="313">
       <c r="A313" t="n">
@@ -15214,7 +15009,6 @@
           <t>Goalim-Moula</t>
         </is>
       </c>
-      <c r="E313" t="inlineStr"/>
       <c r="F313" t="inlineStr">
         <is>
           <t>GOALIM MOVLA</t>
@@ -15260,7 +15054,6 @@
           <t>Goltim</t>
         </is>
       </c>
-      <c r="E314" t="inlineStr"/>
       <c r="F314" t="inlineStr">
         <is>
           <t>GOLTIM</t>
@@ -15361,7 +15154,6 @@
           <t>Malar</t>
         </is>
       </c>
-      <c r="E316" t="inlineStr"/>
       <c r="F316" t="inlineStr">
         <is>
           <t>MALAR</t>
@@ -15407,7 +15199,6 @@
           <t>Mandur</t>
         </is>
       </c>
-      <c r="E317" t="inlineStr"/>
       <c r="F317" t="inlineStr">
         <is>
           <t>MANUR</t>
@@ -15433,6 +15224,11 @@
       <c r="P317" s="2" t="n"/>
       <c r="Q317" s="2" t="n"/>
       <c r="R317" s="2" t="n"/>
+      <c r="V317" t="inlineStr">
+        <is>
+          <t>Mandura</t>
+        </is>
+      </c>
     </row>
     <row r="318">
       <c r="A318" t="n">
@@ -15648,7 +15444,6 @@
           <t>Naroa</t>
         </is>
       </c>
-      <c r="E322" t="inlineStr"/>
       <c r="L322" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -15684,7 +15479,6 @@
           <t>Navelim</t>
         </is>
       </c>
-      <c r="E323" t="inlineStr"/>
       <c r="F323" t="inlineStr">
         <is>
           <t>NAVELI</t>
@@ -15740,7 +15534,6 @@
           <t>Neura-O-Grande</t>
         </is>
       </c>
-      <c r="E324" t="inlineStr"/>
       <c r="F324" t="inlineStr">
         <is>
           <t>NEVRA GRANDE</t>
@@ -15786,7 +15579,6 @@
           <t>Neura-O-Pequeno</t>
         </is>
       </c>
-      <c r="E325" t="inlineStr"/>
       <c r="F325" t="inlineStr">
         <is>
           <t>NEVRA PIKNE</t>
@@ -15832,7 +15624,6 @@
           <t>Panaji</t>
         </is>
       </c>
-      <c r="E326" t="inlineStr"/>
       <c r="L326" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -15948,7 +15739,6 @@
           <t>Siridao</t>
         </is>
       </c>
-      <c r="E329" t="inlineStr"/>
       <c r="F329" t="inlineStr">
         <is>
           <t>SIRIDAO</t>
@@ -15994,7 +15784,6 @@
           <t>Talaulim</t>
         </is>
       </c>
-      <c r="E330" t="inlineStr"/>
       <c r="F330" t="inlineStr">
         <is>
           <t>TALAUIM</t>
@@ -16040,7 +15829,6 @@
           <t>Taleigao</t>
         </is>
       </c>
-      <c r="E331" t="inlineStr"/>
       <c r="F331" t="inlineStr">
         <is>
           <t>DURGAVADO</t>
@@ -16086,7 +15874,6 @@
           <t>Arossim</t>
         </is>
       </c>
-      <c r="E332" t="inlineStr"/>
       <c r="F332" t="inlineStr">
         <is>
           <t>AROSIM</t>
@@ -16137,7 +15924,6 @@
           <t>Cansaulim</t>
         </is>
       </c>
-      <c r="E333" t="inlineStr"/>
       <c r="F333" t="inlineStr">
         <is>
           <t>KANSAVLIM</t>
@@ -16243,7 +16029,6 @@
           <t>Chicolna</t>
         </is>
       </c>
-      <c r="E335" t="inlineStr"/>
       <c r="F335" t="inlineStr">
         <is>
           <t>CHIKOLNA</t>
@@ -16349,7 +16134,6 @@
           <t>Cuelim</t>
         </is>
       </c>
-      <c r="E337" t="inlineStr"/>
       <c r="L337" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -16385,7 +16169,6 @@
           <t>Dabolim</t>
         </is>
       </c>
-      <c r="E338" t="inlineStr"/>
       <c r="F338" t="inlineStr">
         <is>
           <t>IJORSHI</t>
@@ -16446,7 +16229,6 @@
           <t>Issorcim</t>
         </is>
       </c>
-      <c r="E339" t="inlineStr"/>
       <c r="F339" t="inlineStr">
         <is>
           <t>IJORSHI</t>
@@ -16497,7 +16279,6 @@
           <t>Mormugao Port</t>
         </is>
       </c>
-      <c r="E340" t="inlineStr"/>
       <c r="L340" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -16533,7 +16314,6 @@
           <t>Pale</t>
         </is>
       </c>
-      <c r="E341" t="inlineStr"/>
       <c r="F341" t="inlineStr">
         <is>
           <t>PALI</t>
@@ -16584,7 +16364,6 @@
           <t>Quelossim</t>
         </is>
       </c>
-      <c r="E342" t="inlineStr"/>
       <c r="F342" t="inlineStr">
         <is>
           <t>KELOSIM</t>
@@ -16635,7 +16414,6 @@
           <t>Sambhaji</t>
         </is>
       </c>
-      <c r="E343" t="inlineStr"/>
       <c r="L343" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -16731,7 +16509,6 @@
           <t>Sao Jacinto Island</t>
         </is>
       </c>
-      <c r="E345" t="inlineStr"/>
       <c r="L345" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -16767,7 +16544,6 @@
           <t>Sao Jorge Island</t>
         </is>
       </c>
-      <c r="E346" t="inlineStr"/>
       <c r="L346" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -16803,7 +16579,6 @@
           <t>Vadem</t>
         </is>
       </c>
-      <c r="E347" t="inlineStr"/>
       <c r="L347" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -16839,7 +16614,6 @@
           <t>Velsao</t>
         </is>
       </c>
-      <c r="E348" t="inlineStr"/>
       <c r="F348" t="inlineStr">
         <is>
           <t>VELSAVAON</t>
@@ -16885,7 +16659,6 @@
           <t>Adcolna</t>
         </is>
       </c>
-      <c r="E349" t="inlineStr"/>
       <c r="F349" t="inlineStr">
         <is>
           <t>HADKON</t>
@@ -16986,7 +16759,6 @@
           <t>Betora</t>
         </is>
       </c>
-      <c r="E351" t="inlineStr"/>
       <c r="F351" t="inlineStr">
         <is>
           <t>BETORA</t>
@@ -17032,7 +16804,6 @@
           <t>Betqui</t>
         </is>
       </c>
-      <c r="E352" t="inlineStr"/>
       <c r="F352" t="inlineStr">
         <is>
           <t>BETGI</t>
@@ -17083,7 +16854,6 @@
           <t>Boma</t>
         </is>
       </c>
-      <c r="E353" t="inlineStr"/>
       <c r="L353" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -17179,7 +16949,6 @@
           <t>Candepar</t>
         </is>
       </c>
-      <c r="E355" t="inlineStr"/>
       <c r="F355" t="inlineStr">
         <is>
           <t>KHANDEPAR</t>
@@ -17280,7 +17049,6 @@
           <t>Codar</t>
         </is>
       </c>
-      <c r="E357" t="inlineStr"/>
       <c r="F357" t="inlineStr">
         <is>
           <t>KODAR</t>
@@ -17331,7 +17099,6 @@
           <t>Conxem</t>
         </is>
       </c>
-      <c r="E358" t="inlineStr"/>
       <c r="F358" t="inlineStr">
         <is>
           <t>KONSEN</t>
@@ -17382,7 +17149,6 @@
           <t>Cuncoliem</t>
         </is>
       </c>
-      <c r="E359" t="inlineStr"/>
       <c r="F359" t="inlineStr">
         <is>
           <t>KUNKULE</t>
@@ -17428,7 +17194,6 @@
           <t>Cundaim</t>
         </is>
       </c>
-      <c r="E360" t="inlineStr"/>
       <c r="F360" t="inlineStr">
         <is>
           <t>KUNDAI</t>
@@ -17514,7 +17279,6 @@
           <t>Durbhat</t>
         </is>
       </c>
-      <c r="E362" t="inlineStr"/>
       <c r="F362" t="inlineStr">
         <is>
           <t>DURBHAT</t>
@@ -17560,7 +17324,6 @@
           <t>Gangem</t>
         </is>
       </c>
-      <c r="E363" t="inlineStr"/>
       <c r="F363" t="inlineStr">
         <is>
           <t>GOTIAKHADILWADA</t>
@@ -17666,7 +17429,6 @@
           <t>Nirancal</t>
         </is>
       </c>
-      <c r="E365" t="inlineStr"/>
       <c r="F365" t="inlineStr">
         <is>
           <t>KALSAI</t>
@@ -17752,7 +17514,6 @@
           <t>Ponchavadi</t>
         </is>
       </c>
-      <c r="E367" t="inlineStr"/>
       <c r="F367" t="inlineStr">
         <is>
           <t>P A N C H V A D I</t>
@@ -17803,7 +17564,6 @@
           <t>Ponda</t>
         </is>
       </c>
-      <c r="E368" t="inlineStr"/>
       <c r="L368" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -17899,7 +17659,6 @@
           <t>Querim</t>
         </is>
       </c>
-      <c r="E370" t="inlineStr"/>
       <c r="F370" t="inlineStr">
         <is>
           <t>KERI</t>
@@ -17945,7 +17704,6 @@
           <t>Queula</t>
         </is>
       </c>
-      <c r="E371" t="inlineStr"/>
       <c r="L371" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -17981,7 +17739,6 @@
           <t>Savoi-Verem</t>
         </is>
       </c>
-      <c r="E372" t="inlineStr"/>
       <c r="F372" t="inlineStr">
         <is>
           <t>PONDA</t>
@@ -18037,7 +17794,6 @@
           <t>Shiroda</t>
         </is>
       </c>
-      <c r="E373" t="inlineStr"/>
       <c r="F373" t="inlineStr">
         <is>
           <t>SHIRODA</t>
@@ -18088,7 +17844,6 @@
           <t>Telaulim</t>
         </is>
       </c>
-      <c r="E374" t="inlineStr"/>
       <c r="F374" t="inlineStr">
         <is>
           <t>AGAPUR</t>
@@ -18139,7 +17894,6 @@
           <t>Tivrem</t>
         </is>
       </c>
-      <c r="E375" t="inlineStr"/>
       <c r="F375" t="inlineStr">
         <is>
           <t>TIVREN</t>
@@ -18240,7 +17994,6 @@
           <t>Vadi</t>
         </is>
       </c>
-      <c r="E377" t="inlineStr"/>
       <c r="F377" t="inlineStr">
         <is>
           <t>WADI</t>
@@ -18286,7 +18039,6 @@
           <t>Vagurbem</t>
         </is>
       </c>
-      <c r="E378" t="inlineStr"/>
       <c r="F378" t="inlineStr">
         <is>
           <t>KHAJANWADA</t>
@@ -18332,7 +18084,6 @@
           <t>Velinga</t>
         </is>
       </c>
-      <c r="E379" t="inlineStr"/>
       <c r="F379" t="inlineStr">
         <is>
           <t>VELING</t>
@@ -18378,7 +18129,6 @@
           <t>Volvoi</t>
         </is>
       </c>
-      <c r="E380" t="inlineStr"/>
       <c r="F380" t="inlineStr">
         <is>
           <t>VALVAI</t>
@@ -18429,7 +18179,6 @@
           <t>Adsulim</t>
         </is>
       </c>
-      <c r="E381" t="inlineStr"/>
       <c r="F381" t="inlineStr">
         <is>
           <t>ADSULI</t>
@@ -18475,7 +18224,6 @@
           <t>Ambelim</t>
         </is>
       </c>
-      <c r="E382" t="inlineStr"/>
       <c r="L382" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -18511,7 +18259,6 @@
           <t>Aquem-Baixo</t>
         </is>
       </c>
-      <c r="E383" t="inlineStr"/>
       <c r="F383" t="inlineStr">
         <is>
           <t>AKE</t>
@@ -18562,7 +18309,6 @@
           <t>Assolna</t>
         </is>
       </c>
-      <c r="E384" t="inlineStr"/>
       <c r="F384" t="inlineStr">
         <is>
           <t>ASSOLNA</t>
@@ -18653,6 +18399,11 @@
       <c r="P385" s="2" t="n"/>
       <c r="Q385" s="2" t="n"/>
       <c r="R385" s="2" t="n"/>
+      <c r="V385" t="inlineStr">
+        <is>
+          <t>Banavalli</t>
+        </is>
+      </c>
     </row>
     <row r="386">
       <c r="A386" t="n">
@@ -18673,7 +18424,6 @@
           <t>Betalbatim</t>
         </is>
       </c>
-      <c r="E386" t="inlineStr"/>
       <c r="F386" t="inlineStr">
         <is>
           <t>BTALBHATI</t>
@@ -18704,6 +18454,11 @@
       <c r="P386" s="2" t="n"/>
       <c r="Q386" s="2" t="n"/>
       <c r="R386" s="2" t="n"/>
+      <c r="V386" t="inlineStr">
+        <is>
+          <t>Betpatte</t>
+        </is>
+      </c>
     </row>
     <row r="387">
       <c r="A387" t="n">
@@ -18724,7 +18479,6 @@
           <t>Calata</t>
         </is>
       </c>
-      <c r="E387" t="inlineStr"/>
       <c r="F387" t="inlineStr">
         <is>
           <t>GIRIM</t>
@@ -18770,7 +18524,6 @@
           <t>Camurlim</t>
         </is>
       </c>
-      <c r="E388" t="inlineStr"/>
       <c r="F388" t="inlineStr">
         <is>
           <t>KAMARLIM</t>
@@ -18816,7 +18569,6 @@
           <t>Cana</t>
         </is>
       </c>
-      <c r="E389" t="inlineStr"/>
       <c r="F389" t="inlineStr">
         <is>
           <t>KANA</t>
@@ -18867,7 +18619,6 @@
           <t>Carmona</t>
         </is>
       </c>
-      <c r="E390" t="inlineStr"/>
       <c r="F390" t="inlineStr">
         <is>
           <t>KARMANE</t>
@@ -18918,7 +18669,6 @@
           <t>Cavelossim</t>
         </is>
       </c>
-      <c r="E391" t="inlineStr"/>
       <c r="F391" t="inlineStr">
         <is>
           <t>KAVLESI</t>
@@ -18964,7 +18714,6 @@
           <t>Cavorim</t>
         </is>
       </c>
-      <c r="E392" t="inlineStr"/>
       <c r="F392" t="inlineStr">
         <is>
           <t>KAVORIN</t>
@@ -19010,7 +18759,6 @@
           <t>Chandor</t>
         </is>
       </c>
-      <c r="E393" t="inlineStr"/>
       <c r="L393" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -19081,6 +18829,11 @@
       <c r="P394" s="2" t="n"/>
       <c r="Q394" s="2" t="n"/>
       <c r="R394" s="2" t="n"/>
+      <c r="V394" t="inlineStr">
+        <is>
+          <t>Chinchone</t>
+        </is>
+      </c>
     </row>
     <row r="395">
       <c r="A395" t="n">
@@ -19101,7 +18854,6 @@
           <t>Colva</t>
         </is>
       </c>
-      <c r="E395" t="inlineStr"/>
       <c r="F395" t="inlineStr">
         <is>
           <t>KOLVE</t>
@@ -19147,7 +18899,6 @@
           <t>Cuncolim</t>
         </is>
       </c>
-      <c r="E396" t="inlineStr"/>
       <c r="L396" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -19298,7 +19049,6 @@
           <t>Deussua</t>
         </is>
       </c>
-      <c r="E399" t="inlineStr"/>
       <c r="F399" t="inlineStr">
         <is>
           <t>DEVSUA</t>
@@ -19344,7 +19094,6 @@
           <t>Dicarpale</t>
         </is>
       </c>
-      <c r="E400" t="inlineStr"/>
       <c r="F400" t="inlineStr">
         <is>
           <t>DIKARPAL</t>
@@ -19395,7 +19144,6 @@
           <t>Dramapur</t>
         </is>
       </c>
-      <c r="E401" t="inlineStr"/>
       <c r="F401" t="inlineStr">
         <is>
           <t>DRAMAPUR</t>
@@ -19446,7 +19194,6 @@
           <t>Duncolim</t>
         </is>
       </c>
-      <c r="E402" t="inlineStr"/>
       <c r="F402" t="inlineStr">
         <is>
           <t>DHUNKALI</t>
@@ -19492,7 +19239,6 @@
           <t>Gaundaulim</t>
         </is>
       </c>
-      <c r="E403" t="inlineStr"/>
       <c r="F403" t="inlineStr">
         <is>
           <t>GANDAVLI</t>
@@ -19538,7 +19284,6 @@
           <t>Gonsua</t>
         </is>
       </c>
-      <c r="E404" t="inlineStr"/>
       <c r="F404" t="inlineStr">
         <is>
           <t>GANSUA</t>
@@ -19584,7 +19329,6 @@
           <t>Guirdolim</t>
         </is>
       </c>
-      <c r="E405" t="inlineStr"/>
       <c r="F405" t="inlineStr">
         <is>
           <t>GIRDOLIN</t>
@@ -19635,7 +19379,6 @@
           <t>Loutulim</t>
         </is>
       </c>
-      <c r="E406" t="inlineStr"/>
       <c r="F406" t="inlineStr">
         <is>
           <t>RASAAIN</t>
@@ -19681,7 +19424,6 @@
           <t>Macasana</t>
         </is>
       </c>
-      <c r="E407" t="inlineStr"/>
       <c r="F407" t="inlineStr">
         <is>
           <t>MAKAZAN</t>
@@ -19727,7 +19469,6 @@
           <t>Majorda</t>
         </is>
       </c>
-      <c r="E408" t="inlineStr"/>
       <c r="F408" t="inlineStr">
         <is>
           <t>MAJORDA</t>
@@ -19773,7 +19514,6 @@
           <t>Margao</t>
         </is>
       </c>
-      <c r="E409" t="inlineStr"/>
       <c r="L409" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -19789,6 +19529,11 @@
       <c r="P409" s="2" t="n"/>
       <c r="Q409" s="2" t="n"/>
       <c r="R409" s="2" t="n"/>
+      <c r="V409" t="inlineStr">
+        <is>
+          <t>Madgaon</t>
+        </is>
+      </c>
     </row>
     <row r="410">
       <c r="A410" t="n">
@@ -19809,7 +19554,6 @@
           <t>Mulem</t>
         </is>
       </c>
-      <c r="E410" t="inlineStr"/>
       <c r="F410" t="inlineStr">
         <is>
           <t>MULEM</t>
@@ -19855,7 +19599,6 @@
           <t>Nagoa</t>
         </is>
       </c>
-      <c r="E411" t="inlineStr"/>
       <c r="F411" t="inlineStr">
         <is>
           <t>NAGVE</t>
@@ -20021,7 +19764,6 @@
           <t>Orlim</t>
         </is>
       </c>
-      <c r="E414" t="inlineStr"/>
       <c r="F414" t="inlineStr">
         <is>
           <t>URLI</t>
@@ -20067,7 +19809,6 @@
           <t>Paroda</t>
         </is>
       </c>
-      <c r="E415" t="inlineStr"/>
       <c r="F415" t="inlineStr">
         <is>
           <t>PARODA</t>
@@ -20113,7 +19854,6 @@
           <t>Rachol</t>
         </is>
       </c>
-      <c r="E416" t="inlineStr"/>
       <c r="L416" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -20264,7 +20004,6 @@
           <t>Sarzora</t>
         </is>
       </c>
-      <c r="E419" t="inlineStr"/>
       <c r="F419" t="inlineStr">
         <is>
           <t>SARZORA</t>
@@ -20315,7 +20054,6 @@
           <t>Seraulim</t>
         </is>
       </c>
-      <c r="E420" t="inlineStr"/>
       <c r="L420" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -20351,7 +20089,6 @@
           <t>Sernabatim</t>
         </is>
       </c>
-      <c r="E421" t="inlineStr"/>
       <c r="F421" t="inlineStr">
         <is>
           <t>SERNABATIM</t>
@@ -20397,7 +20134,6 @@
           <t>Sirlim</t>
         </is>
       </c>
-      <c r="E422" t="inlineStr"/>
       <c r="L422" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -20433,7 +20169,6 @@
           <t>Talaulim</t>
         </is>
       </c>
-      <c r="E423" t="inlineStr"/>
       <c r="F423" t="inlineStr">
         <is>
           <t>TALAVLI</t>
@@ -20484,7 +20219,6 @@
           <t>Talvorda</t>
         </is>
       </c>
-      <c r="E424" t="inlineStr"/>
       <c r="L424" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -20520,7 +20254,6 @@
           <t>Utorda</t>
         </is>
       </c>
-      <c r="E425" t="inlineStr"/>
       <c r="F425" t="inlineStr">
         <is>
           <t>UTARDA</t>
@@ -20566,7 +20299,6 @@
           <t>Vanelim</t>
         </is>
       </c>
-      <c r="E426" t="inlineStr"/>
       <c r="F426" t="inlineStr">
         <is>
           <t>VANELI</t>
@@ -20672,7 +20404,6 @@
           <t>Varoda</t>
         </is>
       </c>
-      <c r="E428" t="inlineStr"/>
       <c r="L428" t="inlineStr">
         <is>
           <t>No Konkani source</t>
@@ -20708,7 +20439,6 @@
           <t>Velim</t>
         </is>
       </c>
-      <c r="E429" t="inlineStr"/>
       <c r="F429" t="inlineStr">
         <is>
           <t>GORKOMARAD</t>
@@ -20791,7 +20521,7 @@
       <c r="R430" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R430"/>
+  <autoFilter ref="A1:V430"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Village sheet, phase 2: meaning, spellings, vaddos, facts, known for
A village's card now carries where its name comes from (with each
source's hedge and credit), the Gazetteer's 1970 spellings, vaddos,
straight-line distances to Panaji and Margao, parish feasts, zatras and
GI products with their next date, and every source as a link. Built from
confirmed rows of data/credited/ and the review sheet's Gazetteer
columns (read with a small built-in xlsx reader). A Gazetteer Devanagari
form shows on the sheet only, marked Needs review. Villages with two
sourced facts become indexable (23 pages now).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/village_names_review.xlsx
+++ b/data/village_names_review.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Review'!$A$1:$V$430</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Review'!$A$1:$X$430</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -536,7 +536,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V430"/>
+  <dimension ref="A1:X430"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -561,6 +561,8 @@
     <col width="22" customWidth="1" min="20" max="20"/>
     <col width="22" customWidth="1" min="21" max="21"/>
     <col width="22" customWidth="1" min="22" max="22"/>
+    <col width="22" customWidth="1" min="23" max="23"/>
+    <col width="22" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -672,6 +674,16 @@
       <c r="V1" s="1" t="inlineStr">
         <is>
           <t>luis_spelling</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>gazetteer_government</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>gazetteer_soi</t>
         </is>
       </c>
     </row>
@@ -5514,9 +5526,29 @@
       <c r="P107" s="2" t="n"/>
       <c r="Q107" s="2" t="n"/>
       <c r="R107" s="2" t="n"/>
+      <c r="S107" t="inlineStr">
+        <is>
+          <t>हळदोणें</t>
+        </is>
+      </c>
+      <c r="T107" t="inlineStr">
+        <is>
+          <t>Haldone</t>
+        </is>
+      </c>
       <c r="V107" t="inlineStr">
         <is>
           <t>Oidone</t>
+        </is>
+      </c>
+      <c r="W107" t="inlineStr">
+        <is>
+          <t>Aldona</t>
+        </is>
+      </c>
+      <c r="X107" t="inlineStr">
+        <is>
+          <t>Aldona</t>
         </is>
       </c>
     </row>
@@ -20521,7 +20553,7 @@
       <c r="R430" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V430"/>
+  <autoFilter ref="A1:X430"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>